<commit_message>
Publish daily market research dashboard - 2026-05-14 10:55 PDT
</commit_message>
<xml_diff>
--- a/research/daily/data/overnight_watchlist.xlsx
+++ b/research/daily/data/overnight_watchlist.xlsx
@@ -80,42 +80,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>CBRS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fintech/consumer credit</t>
+          <t>AI chip IPO / wafer-scale inference</t>
         </is>
       </c>
       <c r="D2">
-        <v>66.14</v>
+        <v>307.03</v>
       </c>
       <c r="E2">
-        <v>4.57</v>
+        <v>65.96</v>
       </c>
       <c r="F2">
-        <v>4.11</v>
+        <v>65.96</v>
       </c>
       <c r="G2">
-        <v>63.25</v>
+        <v>185.0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>05/14 01:00</t>
+          <t>05/14 06:41</t>
         </is>
       </c>
       <c r="I2">
-        <v>2355298</v>
+        <v>20196751</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>BNPL/consumer-credit beta; sensitive to rates and retail data.</t>
+          <t>Cerebras is a new AI hardware IPO: wafer-scale chips, fast inference, OpenAI/AWS validation, and high first-day IPO volatility.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Strong trend; watch for controlled pullback or VWAP hold.</t>
+          <t>Priority momentum; prefer pullbacks, not chase entries.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -130,25 +130,25 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AI semis</t>
+          <t>AI cloud / neocloud infrastructure</t>
         </is>
       </c>
       <c r="D3">
-        <v>435.47</v>
+        <v>225.59</v>
       </c>
       <c r="E3">
-        <v>4.46</v>
+        <v>8.14</v>
       </c>
       <c r="F3">
-        <v>4.48</v>
+        <v>8.84</v>
       </c>
       <c r="G3">
-        <v>416.88</v>
+        <v>208.6</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -156,11 +156,11 @@
         </is>
       </c>
       <c r="I3">
-        <v>11323915</v>
+        <v>21852982</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Custom silicon/networking beneficiary; Cisco and Nvidia AI-infrastructure read-through.</t>
+          <t>Nebius is a GPU cloud and AI infrastructure capacity play tied to AI compute demand, owned power/site capacity, and enterprise AI workloads.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -180,25 +180,25 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AI cloud</t>
+          <t>AI semis</t>
         </is>
       </c>
       <c r="D4">
-        <v>195.39</v>
+        <v>436.5</v>
       </c>
       <c r="E4">
-        <v>3.11</v>
+        <v>4.71</v>
       </c>
       <c r="F4">
-        <v>2.97</v>
+        <v>4.73</v>
       </c>
       <c r="G4">
-        <v>189.5</v>
+        <v>416.88</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -206,11 +206,11 @@
         </is>
       </c>
       <c r="I4">
-        <v>15851832</v>
+        <v>11402858</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>AI cloud/data-center backlog and capex demand.</t>
+          <t>Custom silicon/networking beneficiary; Cisco and Nvidia AI-infrastructure read-through.</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -230,25 +230,25 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>AFRM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AI software</t>
+          <t>Fintech/consumer credit</t>
         </is>
       </c>
       <c r="D5">
-        <v>133.9236</v>
+        <v>65.98</v>
       </c>
       <c r="E5">
-        <v>2.95</v>
+        <v>4.32</v>
       </c>
       <c r="F5">
-        <v>2.98</v>
+        <v>3.86</v>
       </c>
       <c r="G5">
-        <v>130.09</v>
+        <v>63.25</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -256,11 +256,11 @@
         </is>
       </c>
       <c r="I5">
-        <v>25642659</v>
+        <v>2380490</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>AI software/government-commercial platform momentum; valuation-sensitive.</t>
+          <t>BNPL/consumer-credit beta; sensitive to rates and retail data.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -280,25 +280,25 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AXON</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Public safety tech</t>
+          <t>AI cloud</t>
         </is>
       </c>
       <c r="D6">
-        <v>387.68</v>
+        <v>195.705</v>
       </c>
       <c r="E6">
-        <v>2.9</v>
+        <v>3.27</v>
       </c>
       <c r="F6">
-        <v>2.88</v>
+        <v>3.13</v>
       </c>
       <c r="G6">
-        <v>376.76</v>
+        <v>189.5</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -306,16 +306,16 @@
         </is>
       </c>
       <c r="I6">
-        <v>546276</v>
+        <v>16028734</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Independent public-safety AI/software trend; respect stock-specific strength.</t>
+          <t>AI cloud/data-center backlog and capex demand.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Strong trend; watch for controlled pullback or VWAP hold.</t>
+          <t>Priority momentum; prefer pullbacks, not chase entries.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -330,25 +330,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>AXON</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AI cloud</t>
+          <t>Public safety tech</t>
         </is>
       </c>
       <c r="D7">
-        <v>114.475</v>
+        <v>388.16</v>
       </c>
       <c r="E7">
-        <v>2.37</v>
+        <v>3.03</v>
       </c>
       <c r="F7">
-        <v>2.84</v>
+        <v>3.01</v>
       </c>
       <c r="G7">
-        <v>111.83</v>
+        <v>376.76</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -356,11 +356,11 @@
         </is>
       </c>
       <c r="I7">
-        <v>19108633</v>
+        <v>550114</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>AI compute/cloud capacity theme; high-beta and high-IV.</t>
+          <t>Independent public-safety AI/software trend; respect stock-specific strength.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -380,25 +380,25 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Consumer restaurants</t>
+          <t>AI software</t>
         </is>
       </c>
       <c r="D8">
-        <v>107.41</v>
+        <v>133.9685</v>
       </c>
       <c r="E8">
-        <v>1.42</v>
+        <v>2.98</v>
       </c>
       <c r="F8">
-        <v>1.38</v>
+        <v>3.01</v>
       </c>
       <c r="G8">
-        <v>105.91</v>
+        <v>130.09</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -406,16 +406,16 @@
         </is>
       </c>
       <c r="I8">
-        <v>4312750</v>
+        <v>25777594</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Discretionary consumer, China, labor and margin read-through.</t>
+          <t>AI software/government-commercial platform momentum; valuation-sensitive.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Positive but not decisive; monitor confirmation.</t>
+          <t>Strong trend; watch for controlled pullback or VWAP hold.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -430,25 +430,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mega-cap AI/cloud</t>
+          <t>AI cloud</t>
         </is>
       </c>
       <c r="D9">
-        <v>409.24</v>
+        <v>114.34</v>
       </c>
       <c r="E9">
-        <v>1.34</v>
+        <v>2.24</v>
       </c>
       <c r="F9">
-        <v>0.99</v>
+        <v>2.72</v>
       </c>
       <c r="G9">
-        <v>403.83</v>
+        <v>111.83</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -456,16 +456,16 @@
         </is>
       </c>
       <c r="I9">
-        <v>17231007</v>
+        <v>19210031</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>OpenAI/cloud platform exposure; defensive mega-cap AI lane.</t>
+          <t>AI compute/cloud capacity theme; high-beta and high-IV.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Neutral/watch; needs clearer trend.</t>
+          <t>Strong trend; watch for controlled pullback or VWAP hold.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -480,25 +480,25 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AI semis</t>
+          <t>Consumer restaurants</t>
         </is>
       </c>
       <c r="D10">
-        <v>234.43</v>
+        <v>107.35</v>
       </c>
       <c r="E10">
-        <v>1.15</v>
+        <v>1.36</v>
       </c>
       <c r="F10">
-        <v>3.81</v>
+        <v>1.32</v>
       </c>
       <c r="G10">
-        <v>231.76</v>
+        <v>105.91</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -506,11 +506,11 @@
         </is>
       </c>
       <c r="I10">
-        <v>126697906</v>
+        <v>4400011</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>AI GPU leader; H200/China optionality and direct AI-chip flow.</t>
+          <t>Discretionary consumer, China, labor and margin read-through.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -530,25 +530,25 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Mega-cap AI/cloud</t>
         </is>
       </c>
       <c r="D11">
-        <v>152.62</v>
+        <v>409.2701</v>
       </c>
       <c r="E11">
-        <v>1.06</v>
+        <v>1.35</v>
       </c>
       <c r="F11">
-        <v>0.69</v>
+        <v>1.0</v>
       </c>
       <c r="G11">
-        <v>151.0215</v>
+        <v>403.83</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -556,11 +556,11 @@
         </is>
       </c>
       <c r="I11">
-        <v>4421221</v>
+        <v>17318119</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Oil, energy rotation, inflation hedge and geopolitical beta.</t>
+          <t>OpenAI/cloud platform exposure; defensive mega-cap AI lane.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -580,25 +580,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Energy ETF</t>
+          <t>AI semis</t>
         </is>
       </c>
       <c r="D12">
-        <v>58.075</v>
+        <v>234.648</v>
       </c>
       <c r="E12">
-        <v>1.0</v>
+        <v>1.25</v>
       </c>
       <c r="F12">
-        <v>0.77</v>
+        <v>3.9</v>
       </c>
       <c r="G12">
-        <v>57.5</v>
+        <v>231.76</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -606,16 +606,16 @@
         </is>
       </c>
       <c r="I12">
-        <v>13499217</v>
+        <v>127386252</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Broad energy exposure; cleaner sector gauge than a single oil major.</t>
+          <t>AI GPU leader; H200/China optionality and direct AI-chip flow.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Neutral/watch; needs clearer trend.</t>
+          <t>Positive but not decisive; monitor confirmation.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -639,13 +639,13 @@
         </is>
       </c>
       <c r="D13">
-        <v>435.74</v>
+        <v>435.925</v>
       </c>
       <c r="E13">
-        <v>0.87</v>
+        <v>0.91</v>
       </c>
       <c r="F13">
-        <v>1.12</v>
+        <v>1.17</v>
       </c>
       <c r="G13">
         <v>432.0</v>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="I13">
-        <v>676474</v>
+        <v>685852</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -680,25 +680,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Consumer/travel</t>
+          <t>Energy ETF</t>
         </is>
       </c>
       <c r="D14">
-        <v>133.915</v>
+        <v>58.015</v>
       </c>
       <c r="E14">
-        <v>0.69</v>
+        <v>0.9</v>
       </c>
       <c r="F14">
-        <v>0.71</v>
+        <v>0.67</v>
       </c>
       <c r="G14">
-        <v>133.0</v>
+        <v>57.5</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -706,11 +706,11 @@
         </is>
       </c>
       <c r="I14">
-        <v>1125991</v>
+        <v>13556833</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Travel demand and consumer-spending/rates sensitivity.</t>
+          <t>Broad energy exposure; cleaner sector gauge than a single oil major.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -730,25 +730,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Defensive staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D15">
-        <v>80.785</v>
+        <v>152.3102</v>
       </c>
       <c r="E15">
-        <v>0.59</v>
+        <v>0.85</v>
       </c>
       <c r="F15">
-        <v>0.65</v>
+        <v>0.49</v>
       </c>
       <c r="G15">
-        <v>80.312</v>
+        <v>151.0215</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -756,11 +756,11 @@
         </is>
       </c>
       <c r="I15">
-        <v>4923544</v>
+        <v>4476314</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Defensive consumer staple, dollar/rates and rotation hedge.</t>
+          <t>Oil, energy rotation, inflation hedge and geopolitical beta.</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -780,25 +780,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SMH</t>
+          <t>ABNB</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Semiconductor ETF</t>
+          <t>Consumer/travel</t>
         </is>
       </c>
       <c r="D16">
-        <v>578.4401</v>
+        <v>133.74</v>
       </c>
       <c r="E16">
-        <v>0.45</v>
+        <v>0.56</v>
       </c>
       <c r="F16">
-        <v>1.04</v>
+        <v>0.58</v>
       </c>
       <c r="G16">
-        <v>575.86</v>
+        <v>133.0</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -806,16 +806,16 @@
         </is>
       </c>
       <c r="I16">
-        <v>6184970</v>
+        <v>1139335</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Diversified AI-chip exposure; best broad semiconductor trend gauge.</t>
+          <t>Travel demand and consumer-spending/rates sensitivity.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Positive but not decisive; monitor confirmation.</t>
+          <t>Neutral/watch; needs clearer trend.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -830,25 +830,25 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>SMH</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Social/media</t>
+          <t>Semiconductor ETF</t>
         </is>
       </c>
       <c r="D17">
-        <v>155.26</v>
+        <v>579.07</v>
       </c>
       <c r="E17">
-        <v>0.25</v>
+        <v>0.56</v>
       </c>
       <c r="F17">
-        <v>0.74</v>
+        <v>1.15</v>
       </c>
       <c r="G17">
-        <v>154.88</v>
+        <v>575.86</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -856,16 +856,16 @@
         </is>
       </c>
       <c r="I17">
-        <v>2047986</v>
+        <v>6263017</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Ads, user growth and AI data sentiment.</t>
+          <t>Diversified AI-chip exposure; best broad semiconductor trend gauge.</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Neutral/watch; needs clearer trend.</t>
+          <t>Positive but not decisive; monitor confirmation.</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -880,25 +880,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mega-cap tech</t>
+          <t>Defensive staples</t>
         </is>
       </c>
       <c r="D18">
-        <v>298.14</v>
+        <v>80.655</v>
       </c>
       <c r="E18">
-        <v>0.05</v>
+        <v>0.43</v>
       </c>
       <c r="F18">
-        <v>-0.24</v>
+        <v>0.49</v>
       </c>
       <c r="G18">
-        <v>298.0</v>
+        <v>80.312</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -906,11 +906,11 @@
         </is>
       </c>
       <c r="I18">
-        <v>19401064</v>
+        <v>4960281</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Consumer hardware/services beta; not the cleanest AI-infra mover today.</t>
+          <t>Defensive consumer staple, dollar/rates and rotation hedge.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -930,25 +930,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Mega-cap tech</t>
         </is>
       </c>
       <c r="D19">
-        <v>399.57</v>
+        <v>298.23</v>
       </c>
       <c r="E19">
-        <v>-0.02</v>
+        <v>0.08</v>
       </c>
       <c r="F19">
-        <v>-0.4</v>
+        <v>-0.21</v>
       </c>
       <c r="G19">
-        <v>399.6383</v>
+        <v>298.0</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -956,11 +956,11 @@
         </is>
       </c>
       <c r="I19">
-        <v>3170829</v>
+        <v>19512530</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Managed-care/healthcare policy and utilization sleeve.</t>
+          <t>Consumer hardware/services beta; not the cleanest AI-infra mover today.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -980,25 +980,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>Social/media</t>
         </is>
       </c>
       <c r="D20">
-        <v>87.555</v>
+        <v>154.96</v>
       </c>
       <c r="E20">
-        <v>-0.07</v>
+        <v>0.05</v>
       </c>
       <c r="F20">
-        <v>-0.01</v>
+        <v>0.55</v>
       </c>
       <c r="G20">
-        <v>87.62</v>
+        <v>154.88</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1006,11 +1006,11 @@
         </is>
       </c>
       <c r="I20">
-        <v>14385061</v>
+        <v>2059211</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Consumer subscription/margin story, less tied to AI-chip tape.</t>
+          <t>Ads, user growth and AI data sentiment.</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1030,25 +1030,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cloud/retail</t>
+          <t>AI memory</t>
         </is>
       </c>
       <c r="D21">
-        <v>269.01</v>
+        <v>794.51</v>
       </c>
       <c r="E21">
-        <v>-0.22</v>
+        <v>-0.06</v>
       </c>
       <c r="F21">
-        <v>-0.41</v>
+        <v>-1.13</v>
       </c>
       <c r="G21">
-        <v>269.6097</v>
+        <v>795.0</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1056,11 +1056,11 @@
         </is>
       </c>
       <c r="I21">
-        <v>16382074</v>
+        <v>30456780</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>AWS AI capex plus retail-sales read-through.</t>
+          <t>HBM/memory-cycle exposure; volatile after recent AI-memory rally.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1080,25 +1080,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AI memory</t>
+          <t>Streaming</t>
         </is>
       </c>
       <c r="D22">
-        <v>793.2</v>
+        <v>87.5</v>
       </c>
       <c r="E22">
-        <v>-0.23</v>
+        <v>-0.14</v>
       </c>
       <c r="F22">
-        <v>-1.3</v>
+        <v>-0.07</v>
       </c>
       <c r="G22">
-        <v>795.0</v>
+        <v>87.62</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1106,11 +1106,11 @@
         </is>
       </c>
       <c r="I22">
-        <v>30172552</v>
+        <v>14554813</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>HBM/memory-cycle exposure; volatile after recent AI-memory rally.</t>
+          <t>Consumer subscription/margin story, less tied to AI-chip tape.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1130,25 +1130,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mega-cap AI/ads</t>
+          <t>Cloud/retail</t>
         </is>
       </c>
       <c r="D23">
-        <v>402.37</v>
+        <v>269.175</v>
       </c>
       <c r="E23">
-        <v>-0.26</v>
+        <v>-0.16</v>
       </c>
       <c r="F23">
-        <v>-0.06</v>
+        <v>-0.35</v>
       </c>
       <c r="G23">
-        <v>403.43</v>
+        <v>269.6097</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1156,11 +1156,11 @@
         </is>
       </c>
       <c r="I23">
-        <v>13805799</v>
+        <v>16551574</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>AI/cloud sentiment plus ad-market beta.</t>
+          <t>AWS AI capex plus retail-sales read-through.</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1180,25 +1180,25 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>EV/AI</t>
+          <t>Mega-cap AI/ads</t>
         </is>
       </c>
       <c r="D24">
-        <v>447.0997</v>
+        <v>402.71</v>
       </c>
       <c r="E24">
-        <v>-0.33</v>
+        <v>-0.18</v>
       </c>
       <c r="F24">
-        <v>0.41</v>
+        <v>0.02</v>
       </c>
       <c r="G24">
-        <v>448.6</v>
+        <v>403.43</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1206,11 +1206,11 @@
         </is>
       </c>
       <c r="I24">
-        <v>34512888</v>
+        <v>13994131</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>EV, robotaxi/AI optionality and retail high-beta flow.</t>
+          <t>AI/cloud sentiment plus ad-market beta.</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1239,16 +1239,16 @@
         </is>
       </c>
       <c r="D25">
-        <v>1009.33</v>
+        <v>398.87</v>
       </c>
       <c r="E25">
-        <v>-0.69</v>
+        <v>-0.19</v>
       </c>
       <c r="F25">
-        <v>-0.63</v>
+        <v>-0.57</v>
       </c>
       <c r="G25">
-        <v>1016.36</v>
+        <v>399.6383</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1256,11 +1256,11 @@
         </is>
       </c>
       <c r="I25">
-        <v>912392</v>
+        <v>3183185</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>GLP-1/pharma growth sleeve; useful non-chip diversifier.</t>
+          <t>Managed-care/healthcare policy and utilization sleeve.</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1280,37 +1280,37 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>NMAX</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Speculative media</t>
+          <t>EV/AI</t>
         </is>
       </c>
       <c r="D26">
-        <v>6.71</v>
+        <v>446.69</v>
       </c>
       <c r="E26">
-        <v>-1.18</v>
+        <v>-0.43</v>
       </c>
       <c r="F26">
-        <v>-1.47</v>
+        <v>0.32</v>
       </c>
       <c r="G26">
-        <v>6.79</v>
+        <v>448.6</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>05/14 01:01</t>
+          <t>05/14 01:00</t>
         </is>
       </c>
       <c r="I26">
-        <v>607594</v>
+        <v>34756780</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>High-IV media/speculative flow; data quality and liquidity need caution.</t>
+          <t>EV, robotaxi/AI optionality and retail high-beta flow.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -1330,25 +1330,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CRCL</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Crypto/fintech</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D27">
-        <v>124.905</v>
+        <v>1008.596</v>
       </c>
       <c r="E27">
-        <v>-1.34</v>
+        <v>-0.76</v>
       </c>
       <c r="F27">
-        <v>-1.32</v>
+        <v>-0.7</v>
       </c>
       <c r="G27">
-        <v>126.6</v>
+        <v>1016.36</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1356,11 +1356,11 @@
         </is>
       </c>
       <c r="I27">
-        <v>16999392</v>
+        <v>920571</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Crypto beta and high-IV speculative flow.</t>
+          <t>GLP-1/pharma growth sleeve; useful non-chip diversifier.</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -1380,25 +1380,25 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>NEM</t>
+          <t>CRCL</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gold/mining</t>
+          <t>Crypto/fintech</t>
         </is>
       </c>
       <c r="D28">
-        <v>116.715</v>
+        <v>125.205</v>
       </c>
       <c r="E28">
-        <v>-1.77</v>
+        <v>-1.1</v>
       </c>
       <c r="F28">
-        <v>-1.89</v>
+        <v>-1.08</v>
       </c>
       <c r="G28">
-        <v>118.815</v>
+        <v>126.6</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1406,11 +1406,11 @@
         </is>
       </c>
       <c r="I28">
-        <v>2365989</v>
+        <v>17172301</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Gold, real-rate, dollar and inflation hedge.</t>
+          <t>Crypto beta and high-IV speculative flow.</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -1430,45 +1430,145 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>NMAX</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Speculative media</t>
+        </is>
+      </c>
+      <c r="D29">
+        <v>6.71</v>
+      </c>
+      <c r="E29">
+        <v>-1.18</v>
+      </c>
+      <c r="F29">
+        <v>-1.47</v>
+      </c>
+      <c r="G29">
+        <v>6.79</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>05/14 01:01</t>
+        </is>
+      </c>
+      <c r="I29">
+        <v>611485</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>High-IV media/speculative flow; data quality and liquidity need caution.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Neutral/watch; needs clearer trend.</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>INTC</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Semis/foundry</t>
         </is>
       </c>
-      <c r="D29">
-        <v>115.71</v>
-      </c>
-      <c r="E29">
-        <v>-1.77</v>
-      </c>
-      <c r="F29">
-        <v>-3.81</v>
-      </c>
-      <c r="G29">
+      <c r="D30">
+        <v>115.83</v>
+      </c>
+      <c r="E30">
+        <v>-1.67</v>
+      </c>
+      <c r="F30">
+        <v>-3.71</v>
+      </c>
+      <c r="G30">
         <v>117.8</v>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>05/14 01:00</t>
         </is>
       </c>
-      <c r="I29">
-        <v>81173525</v>
-      </c>
-      <c r="J29" t="inlineStr">
+      <c r="I30">
+        <v>81834497</v>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>Foundry-turnaround debate; recent pullback on yield/loss concerns.</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>Neutral/watch; needs clearer trend.</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NEM</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Gold/mining</t>
+        </is>
+      </c>
+      <c r="D31">
+        <v>116.63</v>
+      </c>
+      <c r="E31">
+        <v>-1.84</v>
+      </c>
+      <c r="F31">
+        <v>-1.96</v>
+      </c>
+      <c r="G31">
+        <v>118.815</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>05/14 01:00</t>
+        </is>
+      </c>
+      <c r="I31">
+        <v>2385578</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Gold, real-rate, dollar and inflation hedge.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Neutral/watch; needs clearer trend.</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2110,645 +2210,715 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AI cloud</t>
+          <t>AI cloud / neocloud infrastructure</t>
         </is>
       </c>
       <c r="C15"/>
       <c r="D15">
-        <v>190.2</v>
+        <v>209.5</v>
       </c>
       <c r="E15">
-        <v>189.52</v>
+        <v>206.0</v>
       </c>
       <c r="F15">
-        <v>190.0</v>
+        <v>206.35</v>
       </c>
       <c r="G15">
-        <v>190.41</v>
+        <v>206.33</v>
       </c>
       <c r="H15">
-        <v>190.4</v>
+        <v>212.0</v>
       </c>
       <c r="I15">
-        <v>188.66</v>
+        <v>208.5</v>
       </c>
       <c r="J15">
-        <v>195.02</v>
+        <v>223.17</v>
       </c>
       <c r="K15">
-        <v>199.1901</v>
+        <v>229.7</v>
       </c>
       <c r="L15">
-        <v>198.1</v>
+        <v>232.8</v>
       </c>
       <c r="M15">
-        <v>195.865</v>
+        <v>226.595</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AI software</t>
+          <t>AI cloud</t>
         </is>
       </c>
       <c r="C16"/>
       <c r="D16">
-        <v>130.2</v>
+        <v>190.2</v>
       </c>
       <c r="E16">
-        <v>130.4</v>
+        <v>189.52</v>
       </c>
       <c r="F16">
-        <v>130.76</v>
+        <v>190.0</v>
       </c>
       <c r="G16">
-        <v>130.1948</v>
+        <v>190.41</v>
       </c>
       <c r="H16">
-        <v>130.22</v>
+        <v>190.4</v>
       </c>
       <c r="I16">
-        <v>131.229</v>
+        <v>188.66</v>
       </c>
       <c r="J16">
-        <v>131.93</v>
+        <v>195.02</v>
       </c>
       <c r="K16">
-        <v>132.67</v>
+        <v>199.1901</v>
       </c>
       <c r="L16">
-        <v>133.345</v>
+        <v>198.1</v>
       </c>
       <c r="M16">
-        <v>133.47</v>
+        <v>195.865</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Social/media</t>
+          <t>AI software</t>
         </is>
       </c>
       <c r="C17"/>
       <c r="D17">
-        <v>155.68</v>
+        <v>130.2</v>
       </c>
       <c r="E17">
-        <v>155.2</v>
+        <v>130.4</v>
       </c>
       <c r="F17">
-        <v>154.07</v>
+        <v>130.76</v>
       </c>
       <c r="G17">
-        <v>155.29</v>
+        <v>130.1948</v>
       </c>
       <c r="H17">
-        <v>154.99</v>
+        <v>130.22</v>
       </c>
       <c r="I17">
-        <v>155.775</v>
+        <v>131.229</v>
       </c>
       <c r="J17">
-        <v>152.065</v>
+        <v>131.93</v>
       </c>
       <c r="K17">
-        <v>154.995</v>
+        <v>132.67</v>
       </c>
       <c r="L17">
-        <v>155.99</v>
+        <v>133.345</v>
       </c>
       <c r="M17">
-        <v>155.11</v>
+        <v>133.47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SMH</t>
+          <t>CBRS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Semiconductor ETF</t>
+          <t>AI chip IPO / wafer-scale inference</t>
         </is>
       </c>
       <c r="C18"/>
-      <c r="D18">
-        <v>574.74</v>
-      </c>
-      <c r="E18">
-        <v>571.13</v>
-      </c>
-      <c r="F18">
-        <v>571.05</v>
-      </c>
-      <c r="G18">
-        <v>571.61</v>
-      </c>
-      <c r="H18">
-        <v>573.0</v>
-      </c>
-      <c r="I18">
-        <v>568.4715</v>
-      </c>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18"/>
+      <c r="I18"/>
       <c r="J18">
-        <v>576.705</v>
-      </c>
-      <c r="K18">
-        <v>580.25</v>
-      </c>
-      <c r="L18">
-        <v>579.35</v>
-      </c>
+        <v>185.0</v>
+      </c>
+      <c r="K18"/>
+      <c r="L18"/>
       <c r="M18">
-        <v>575.68</v>
+        <v>328.57</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SPOT</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Consumer/subscription</t>
+          <t>Social/media</t>
         </is>
       </c>
       <c r="C19"/>
       <c r="D19">
-        <v>430.99</v>
+        <v>155.68</v>
       </c>
       <c r="E19">
-        <v>433.97</v>
+        <v>155.2</v>
       </c>
       <c r="F19">
-        <v>431.02</v>
+        <v>154.07</v>
       </c>
       <c r="G19">
-        <v>425.5562</v>
+        <v>155.29</v>
       </c>
       <c r="H19">
-        <v>431.99</v>
+        <v>154.99</v>
       </c>
       <c r="I19">
-        <v>437.8585</v>
+        <v>155.775</v>
       </c>
       <c r="J19">
-        <v>437.03</v>
+        <v>152.065</v>
       </c>
       <c r="K19">
-        <v>438.61</v>
+        <v>154.995</v>
       </c>
       <c r="L19">
-        <v>437.205</v>
+        <v>155.99</v>
       </c>
       <c r="M19">
-        <v>436.17</v>
+        <v>155.11</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>SMH</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EV/AI</t>
+          <t>Semiconductor ETF</t>
         </is>
       </c>
       <c r="C20"/>
       <c r="D20">
-        <v>448.66</v>
+        <v>574.74</v>
       </c>
       <c r="E20">
-        <v>446.88</v>
+        <v>571.13</v>
       </c>
       <c r="F20">
-        <v>448.37</v>
+        <v>571.05</v>
       </c>
       <c r="G20">
-        <v>450.1899</v>
+        <v>571.61</v>
       </c>
       <c r="H20">
-        <v>449.9</v>
+        <v>573.0</v>
       </c>
       <c r="I20">
-        <v>445.329</v>
+        <v>568.4715</v>
       </c>
       <c r="J20">
-        <v>442.8899</v>
+        <v>576.705</v>
       </c>
       <c r="K20">
-        <v>446.81</v>
+        <v>580.25</v>
       </c>
       <c r="L20">
-        <v>449.035</v>
+        <v>579.35</v>
       </c>
       <c r="M20">
-        <v>445.0593</v>
+        <v>575.68</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NMAX</t>
+          <t>SPOT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Speculative media</t>
+          <t>Consumer/subscription</t>
         </is>
       </c>
       <c r="C21"/>
       <c r="D21">
-        <v>6.79</v>
+        <v>430.99</v>
       </c>
       <c r="E21">
-        <v>6.74</v>
+        <v>433.97</v>
       </c>
       <c r="F21">
-        <v>6.79</v>
+        <v>431.02</v>
       </c>
       <c r="G21">
-        <v>6.78</v>
+        <v>425.5562</v>
       </c>
       <c r="H21">
-        <v>6.81</v>
+        <v>431.99</v>
       </c>
       <c r="I21">
-        <v>6.81</v>
+        <v>437.8585</v>
       </c>
       <c r="J21">
-        <v>6.83</v>
+        <v>437.03</v>
       </c>
       <c r="K21">
-        <v>6.87</v>
+        <v>438.61</v>
       </c>
       <c r="L21">
-        <v>6.79</v>
+        <v>437.205</v>
       </c>
       <c r="M21">
-        <v>6.7</v>
+        <v>436.17</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Defensive staples</t>
+          <t>EV/AI</t>
         </is>
       </c>
       <c r="C22"/>
       <c r="D22">
-        <v>80.29</v>
+        <v>448.66</v>
       </c>
       <c r="E22">
-        <v>80.2</v>
+        <v>446.88</v>
       </c>
       <c r="F22">
-        <v>80.3</v>
+        <v>448.37</v>
       </c>
       <c r="G22">
-        <v>80.21</v>
+        <v>450.1899</v>
       </c>
       <c r="H22">
-        <v>80.51</v>
+        <v>449.9</v>
       </c>
       <c r="I22">
-        <v>80.515</v>
+        <v>445.329</v>
       </c>
       <c r="J22">
-        <v>80.38</v>
+        <v>442.8899</v>
       </c>
       <c r="K22">
-        <v>80.56</v>
+        <v>446.81</v>
       </c>
       <c r="L22">
-        <v>80.78</v>
+        <v>449.035</v>
       </c>
       <c r="M22">
-        <v>80.66</v>
+        <v>445.0593</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>NMAX</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fintech/consumer credit</t>
+          <t>Speculative media</t>
         </is>
       </c>
       <c r="C23"/>
       <c r="D23">
-        <v>64.3</v>
+        <v>6.79</v>
       </c>
       <c r="E23">
-        <v>63.4</v>
+        <v>6.74</v>
       </c>
       <c r="F23">
-        <v>63.84</v>
+        <v>6.79</v>
       </c>
       <c r="G23">
-        <v>64.3999</v>
+        <v>6.78</v>
       </c>
       <c r="H23">
-        <v>63.66</v>
+        <v>6.81</v>
       </c>
       <c r="I23">
-        <v>64.44</v>
+        <v>6.81</v>
       </c>
       <c r="J23">
-        <v>65.52</v>
+        <v>6.83</v>
       </c>
       <c r="K23">
-        <v>66.05</v>
+        <v>6.87</v>
       </c>
       <c r="L23">
-        <v>66.35</v>
+        <v>6.79</v>
       </c>
       <c r="M23">
-        <v>66.1075</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Consumer restaurants</t>
+          <t>Defensive staples</t>
         </is>
       </c>
       <c r="C24"/>
       <c r="D24">
-        <v>105.92</v>
+        <v>80.29</v>
       </c>
       <c r="E24">
-        <v>107.19</v>
+        <v>80.2</v>
       </c>
       <c r="F24">
-        <v>107.21</v>
+        <v>80.3</v>
       </c>
       <c r="G24">
-        <v>107.21</v>
+        <v>80.21</v>
       </c>
       <c r="H24">
-        <v>107.4</v>
+        <v>80.51</v>
       </c>
       <c r="I24">
-        <v>108.06</v>
+        <v>80.515</v>
       </c>
       <c r="J24">
-        <v>107.75</v>
+        <v>80.38</v>
       </c>
       <c r="K24">
-        <v>107.794</v>
+        <v>80.56</v>
       </c>
       <c r="L24">
-        <v>107.65</v>
+        <v>80.78</v>
       </c>
       <c r="M24">
-        <v>107.07</v>
+        <v>80.66</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>AFRM</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Semis/foundry</t>
+          <t>Fintech/consumer credit</t>
         </is>
       </c>
       <c r="C25"/>
       <c r="D25">
-        <v>117.13</v>
+        <v>64.3</v>
       </c>
       <c r="E25">
-        <v>116.1858</v>
+        <v>63.4</v>
       </c>
       <c r="F25">
-        <v>115.97</v>
+        <v>63.84</v>
       </c>
       <c r="G25">
-        <v>115.99</v>
+        <v>64.3999</v>
       </c>
       <c r="H25">
-        <v>116.255</v>
+        <v>63.66</v>
       </c>
       <c r="I25">
-        <v>114.0205</v>
+        <v>64.44</v>
       </c>
       <c r="J25">
-        <v>114.75</v>
+        <v>65.52</v>
       </c>
       <c r="K25">
-        <v>116.205</v>
+        <v>66.05</v>
       </c>
       <c r="L25">
-        <v>116.66</v>
+        <v>66.35</v>
       </c>
       <c r="M25">
-        <v>114.99</v>
+        <v>66.1075</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer restaurants</t>
         </is>
       </c>
       <c r="C26"/>
       <c r="D26">
-        <v>1014.86</v>
+        <v>105.92</v>
       </c>
       <c r="E26">
-        <v>1010.99</v>
+        <v>107.19</v>
       </c>
       <c r="F26">
-        <v>1024.0</v>
+        <v>107.21</v>
       </c>
       <c r="G26">
-        <v>1020.0</v>
+        <v>107.21</v>
       </c>
       <c r="H26">
-        <v>1015.2022</v>
+        <v>107.4</v>
       </c>
       <c r="I26">
-        <v>1010.35</v>
+        <v>108.06</v>
       </c>
       <c r="J26">
-        <v>1006.365</v>
+        <v>107.75</v>
       </c>
       <c r="K26">
-        <v>1001.5</v>
+        <v>107.794</v>
       </c>
       <c r="L26">
-        <v>1006.1999</v>
+        <v>107.65</v>
       </c>
       <c r="M26">
-        <v>1009.53</v>
+        <v>107.07</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Semis/foundry</t>
         </is>
       </c>
       <c r="C27"/>
       <c r="D27">
-        <v>399.14</v>
+        <v>117.13</v>
       </c>
       <c r="E27">
-        <v>400.03</v>
+        <v>116.1858</v>
       </c>
       <c r="F27">
-        <v>401.67</v>
+        <v>115.97</v>
       </c>
       <c r="G27">
-        <v>401.15</v>
+        <v>115.99</v>
       </c>
       <c r="H27">
-        <v>401.86</v>
+        <v>116.255</v>
       </c>
       <c r="I27">
-        <v>400.23</v>
+        <v>114.0205</v>
       </c>
       <c r="J27">
-        <v>397.251</v>
+        <v>114.75</v>
       </c>
       <c r="K27">
-        <v>398.385</v>
+        <v>116.205</v>
       </c>
       <c r="L27">
-        <v>399.065</v>
+        <v>116.66</v>
       </c>
       <c r="M27">
-        <v>398.665</v>
+        <v>114.99</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="C28"/>
       <c r="D28">
-        <v>150.99</v>
+        <v>1014.86</v>
       </c>
       <c r="E28">
-        <v>151.37</v>
+        <v>1010.99</v>
       </c>
       <c r="F28">
-        <v>151.33</v>
+        <v>1024.0</v>
       </c>
       <c r="G28">
-        <v>151.51</v>
+        <v>1020.0</v>
       </c>
       <c r="H28">
-        <v>151.57</v>
+        <v>1015.2022</v>
       </c>
       <c r="I28">
-        <v>152.0</v>
+        <v>1010.35</v>
       </c>
       <c r="J28">
-        <v>152.75</v>
+        <v>1006.365</v>
       </c>
       <c r="K28">
-        <v>151.95</v>
+        <v>1001.5</v>
       </c>
       <c r="L28">
-        <v>152.26</v>
+        <v>1006.1999</v>
       </c>
       <c r="M28">
-        <v>152.51</v>
+        <v>1009.53</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Energy ETF</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="C29"/>
       <c r="D29">
+        <v>399.14</v>
+      </c>
+      <c r="E29">
+        <v>400.03</v>
+      </c>
+      <c r="F29">
+        <v>401.67</v>
+      </c>
+      <c r="G29">
+        <v>401.15</v>
+      </c>
+      <c r="H29">
+        <v>401.86</v>
+      </c>
+      <c r="I29">
+        <v>400.23</v>
+      </c>
+      <c r="J29">
+        <v>397.251</v>
+      </c>
+      <c r="K29">
+        <v>398.385</v>
+      </c>
+      <c r="L29">
+        <v>399.065</v>
+      </c>
+      <c r="M29">
+        <v>398.665</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C30"/>
+      <c r="D30">
+        <v>150.99</v>
+      </c>
+      <c r="E30">
+        <v>151.37</v>
+      </c>
+      <c r="F30">
+        <v>151.33</v>
+      </c>
+      <c r="G30">
+        <v>151.51</v>
+      </c>
+      <c r="H30">
+        <v>151.57</v>
+      </c>
+      <c r="I30">
+        <v>152.0</v>
+      </c>
+      <c r="J30">
+        <v>152.75</v>
+      </c>
+      <c r="K30">
+        <v>151.95</v>
+      </c>
+      <c r="L30">
+        <v>152.26</v>
+      </c>
+      <c r="M30">
+        <v>152.51</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Energy ETF</t>
+        </is>
+      </c>
+      <c r="C31"/>
+      <c r="D31">
         <v>57.5127</v>
       </c>
-      <c r="E29">
+      <c r="E31">
         <v>57.61</v>
       </c>
-      <c r="F29">
+      <c r="F31">
         <v>57.56</v>
       </c>
-      <c r="G29">
+      <c r="G31">
         <v>57.63</v>
       </c>
-      <c r="H29">
+      <c r="H31">
         <v>57.61</v>
       </c>
-      <c r="I29">
+      <c r="I31">
         <v>57.68</v>
       </c>
-      <c r="J29">
+      <c r="J31">
         <v>57.87</v>
       </c>
-      <c r="K29">
+      <c r="K31">
         <v>57.695</v>
       </c>
-      <c r="L29">
+      <c r="L31">
         <v>57.965</v>
       </c>
-      <c r="M29">
+      <c r="M31">
         <v>58.06</v>
       </c>
     </row>
@@ -2767,7 +2937,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-05-14T10:51:25-07:00</t>
+          <t>2026-05-14T10:55:48-07:00</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2949,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00-07:00 to 2026-05-14T10:51:25-07:00</t>
+          <t>2026-05-14T00:00:00-07:00 to 2026-05-14T10:55:48-07:00</t>
         </is>
       </c>
     </row>
@@ -2799,68 +2969,810 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Caveats</t>
+          <t>Category Map</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Public Yahoo data usually begins at 1:00 AM PT for U.S. equities; Schwab/thinkorswim 24-hour marks may not be fully reconstructable unless sampled live.</t>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Names</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Avg % Since Baseline</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Leader %</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>How To Read It</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Recommendations are research signals, not personalized buy/sell instructions.</t>
+          <t>AI chip IPO / wafer-scale inference</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>65.96</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CBRS</t>
+        </is>
+      </c>
+      <c r="E7">
+        <v>65.96</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Fresh IPO risk/reward; first-day price discovery can be violent, so judge by base-building and volume, not excitement alone.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>For entries, use the live platform chart, bid/ask spread, VWAP, and your day-trade/risk limits before acting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
+          <t>AI cloud / neocloud infrastructure</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>8.14</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>8.14</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>GPU cloud and AI compute-capacity exposure; more volatile than mega-cap cloud but tied to the same demand wave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fintech/consumer credit</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>4.32</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>AFRM</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>4.32</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Public safety tech</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>3.03</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>AXON</t>
+        </is>
+      </c>
+      <c r="E10">
+        <v>3.03</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Yahoo Finance chart API</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://query1.finance.yahoo.com/v8/finance/chart/</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Minute-level public quote history used for hourly marks where available.</t>
+          <t>AI semis</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>2.98</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="E11">
+        <v>4.71</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Direct chip/AI hardware exposure; strongest when NVDA, AVGO, and SMH confirm together.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>AI software</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>2.98</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="E12">
+        <v>2.98</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Application/software AI momentum; highly valuation-sensitive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AI cloud</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13">
+        <v>2.75</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="E13">
+        <v>3.27</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Cloud infrastructure capacity and AI hosting demand; watch ORCL/CRWV/NBIS for compute-spend breadth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Consumer restaurants</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>1.36</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SBUX</t>
+        </is>
+      </c>
+      <c r="E14">
+        <v>1.36</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mega-cap AI/cloud</t>
+        </is>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>1.35</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="E15">
+        <v>1.35</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Consumer/subscription</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>0.91</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="E16">
+        <v>0.91</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Energy ETF</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>0.9</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="E17">
+        <v>0.9</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Broad energy sector gauge; helps separate stock-specific oil moves from sector rotation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>0.85</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="E18">
+        <v>0.85</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Oil/inflation/geopolitical hedge; confirms whether macro money is rotating away from duration tech.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Consumer/travel</t>
+        </is>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>0.56</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ABNB</t>
+        </is>
+      </c>
+      <c r="E19">
+        <v>0.56</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Semiconductor ETF</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>0.56</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="E20">
+        <v>0.56</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Broad chip confirmation gauge; cleaner than single-stock chip exposure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Defensive staples</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>0.43</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E21">
+        <v>0.43</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mega-cap tech</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>0.08</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="E22">
+        <v>0.08</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Social/media</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>0.05</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="E23">
+        <v>0.05</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AI memory</t>
+        </is>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>-0.06</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="E24">
+        <v>-0.06</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Streaming</t>
+        </is>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>-0.14</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E25">
+        <v>-0.14</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cloud/retail</t>
+        </is>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>-0.16</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="E26">
+        <v>-0.16</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mega-cap AI/ads</t>
+        </is>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>-0.18</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="E27">
+        <v>-0.18</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EV/AI</t>
+        </is>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>-0.43</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="E28">
+        <v>-0.43</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29">
+        <v>-0.47</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="E29">
+        <v>-0.19</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Defensive/growth diversifier; useful when chip momentum fades or policy headlines drive rotation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Crypto/fintech</t>
+        </is>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30">
+        <v>-1.1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CRCL</t>
+        </is>
+      </c>
+      <c r="E30">
+        <v>-1.1</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Speculative media</t>
+        </is>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31">
+        <v>-1.18</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>NMAX</t>
+        </is>
+      </c>
+      <c r="E31">
+        <v>-1.18</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Semis/foundry</t>
+        </is>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32">
+        <v>-1.67</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="E32">
+        <v>-1.67</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Gold/mining</t>
+        </is>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>-1.84</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>NEM</t>
+        </is>
+      </c>
+      <c r="E33">
+        <v>-1.84</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Single-name or sector-specific trend; use the hourly marks to confirm whether strength is persistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Caveats</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Public Yahoo data usually begins at 1:00 AM PT for U.S. equities; Schwab/thinkorswim 24-hour marks may not be fully reconstructable unless sampled live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Recommendations are research signals, not personalized buy/sell instructions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>For entries, use the live platform chart, bid/ask spread, VWAP, and your day-trade/risk limits before acting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Yahoo Finance chart API</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://query1.finance.yahoo.com/v8/finance/chart/</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Minute-level public quote history used for hourly marks where available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>Daily dashboard market thesis</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>index.html</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>AI infrastructure bid versus macro/rates gate used for interpretation.</t>
         </is>

</xml_diff>